<commit_message>
updated ski resort data
</commit_message>
<xml_diff>
--- a/ski_resort_data.xlsx
+++ b/ski_resort_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a90b1d0dba7937b6/Desktop/Documents/website/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="152" documentId="11_85381FD58F79A8D366075C52F37BD2729A4B12E6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C6AE1BDC-0529-4BB3-90B7-E6F0B14BBB96}"/>
+  <xr:revisionPtr revIDLastSave="153" documentId="11_85381FD58F79A8D366075C52F37BD2729A4B12E6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7B0047C1-82EB-4455-BEAD-DC3365885C67}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1812,7 +1812,7 @@
         <v>4</v>
       </c>
       <c r="R19" t="s">
-        <v>74</v>
+        <v>18</v>
       </c>
       <c r="S19" s="3" t="s">
         <v>98</v>

</xml_diff>